<commit_message>
Trim Daily Log to only the fields that feed a formula
Drop-off Rate %, comment-quality count, DM response time,
click-throughs, and a screenshot flag never fed Hook Bank, Format
Comparison, or Boss Presentation Summary -- they were 5 of 18 columns
of pure daily typing with no automated payoff. Cut to the 7 data
columns that actually drive the analysis, plus Notes for anything
qualitative. Re-verified against the same synthetic dataset used
before the change: identical output (3050 views, 17 DMs, Carousel
winning, V8 top hook), confirming the trim only removed unused
columns and didn't change any result.

Synced the checklist (posting_checklist.md and the mobile hub) to
match -- 11 items down to 10, no more referencing columns that no
longer exist.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AgaN3EJLBSBRTVA9kYmAXk
</commit_message>
<xml_diff>
--- a/campaign/Goaldenway_Boathouse_Tracker.xlsx
+++ b/campaign/Goaldenway_Boathouse_Tracker.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="120">
   <si>
     <t xml:space="preserve">Goaldenway x The Boat House — 30-Day IG Campaign Tracker</t>
   </si>
@@ -92,6 +92,9 @@
     <t xml:space="preserve">- Repeatable? cells and the Format Comparison Winner row are now color-coded (green/amber/red) via conditional formatting, so status is visible at a glance without reading text -- useful when checking this on a phone.</t>
   </si>
   <si>
+    <t xml:space="preserve">- Daily Log was trimmed from 18 columns to 13: Drop-off Rate %, Comments-Buying-Signal count, DM Response Time, Click-throughs, and Screenshot Taken were cut because none of them fed a single formula anywhere in this workbook -- they were just extra typing every day for no automated payoff. If something from those is worth flagging on a given day (a slow DM reply, a standout comment), put it in Notes. The 'reply within 5 min' and 'screenshot Insights' reminders now live as checkboxes in the mobile campaign hub instead.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hook ID</t>
   </si>
   <si>
@@ -281,9 +284,6 @@
     <t xml:space="preserve">Watch Time %</t>
   </si>
   <si>
-    <t xml:space="preserve">Drop-off Rate %</t>
-  </si>
-  <si>
     <t xml:space="preserve">Likes</t>
   </si>
   <si>
@@ -297,18 +297,6 @@
   </si>
   <si>
     <t xml:space="preserve">Comments (Total)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comments - Buying Signal (#)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DM Response Time (min, avg)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Click-throughs to page/tag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Screenshot Taken (Y/N)</t>
   </si>
   <si>
     <t xml:space="preserve">Notes</t>
@@ -956,7 +944,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="100"/>
@@ -1070,6 +1058,11 @@
     <row r="26" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1103,42 +1096,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D2" s="6" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A2)</f>
@@ -1153,11 +1146,11 @@
         <v/>
       </c>
       <c r="G2" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A2,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A2,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H2" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A2,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A2,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I2" s="6" t="str">
@@ -1167,13 +1160,13 @@
     </row>
     <row r="3" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D3" s="9" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A3)</f>
@@ -1188,11 +1181,11 @@
         <v/>
       </c>
       <c r="G3" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A3,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A3,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H3" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A3,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A3,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I3" s="9" t="str">
@@ -1202,13 +1195,13 @@
     </row>
     <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D4" s="6" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A4)</f>
@@ -1223,11 +1216,11 @@
         <v/>
       </c>
       <c r="G4" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A4,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A4,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H4" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A4,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A4,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I4" s="6" t="str">
@@ -1237,13 +1230,13 @@
     </row>
     <row r="5" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D5" s="9" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A5)</f>
@@ -1258,11 +1251,11 @@
         <v/>
       </c>
       <c r="G5" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A5,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A5,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H5" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A5,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A5,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I5" s="9" t="str">
@@ -1272,13 +1265,13 @@
     </row>
     <row r="6" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A6)</f>
@@ -1293,11 +1286,11 @@
         <v/>
       </c>
       <c r="G6" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A6,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A6,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H6" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A6,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A6,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I6" s="6" t="str">
@@ -1307,13 +1300,13 @@
     </row>
     <row r="7" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A7)</f>
@@ -1328,11 +1321,11 @@
         <v/>
       </c>
       <c r="G7" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A7,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A7,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H7" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A7,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A7,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I7" s="9" t="str">
@@ -1342,13 +1335,13 @@
     </row>
     <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A8)</f>
@@ -1363,11 +1356,11 @@
         <v/>
       </c>
       <c r="G8" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A8,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A8,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H8" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A8,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A8,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I8" s="6" t="str">
@@ -1377,13 +1370,13 @@
     </row>
     <row r="9" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A9)</f>
@@ -1398,11 +1391,11 @@
         <v/>
       </c>
       <c r="G9" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A9,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A9,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H9" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A9,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A9,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I9" s="9" t="str">
@@ -1412,13 +1405,13 @@
     </row>
     <row r="10" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D10" s="6" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A10)</f>
@@ -1433,11 +1426,11 @@
         <v/>
       </c>
       <c r="G10" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A10,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A10,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H10" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A10,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A10,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I10" s="6" t="str">
@@ -1447,13 +1440,13 @@
     </row>
     <row r="11" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D11" s="9" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A11)</f>
@@ -1468,11 +1461,11 @@
         <v/>
       </c>
       <c r="G11" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A11,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A11,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H11" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A11,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A11,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I11" s="9" t="str">
@@ -1482,13 +1475,13 @@
     </row>
     <row r="12" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D12" s="6" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A12)</f>
@@ -1503,11 +1496,11 @@
         <v/>
       </c>
       <c r="G12" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A12,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A12,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H12" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A12,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A12,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I12" s="6" t="str">
@@ -1517,13 +1510,13 @@
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D13" s="9" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A13)</f>
@@ -1538,11 +1531,11 @@
         <v/>
       </c>
       <c r="G13" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A13,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A13,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H13" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A13,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A13,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I13" s="9" t="str">
@@ -1552,13 +1545,13 @@
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D14" s="6" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A14)</f>
@@ -1573,11 +1566,11 @@
         <v/>
       </c>
       <c r="G14" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A14,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A14,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H14" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A14,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A14,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I14" s="6" t="str">
@@ -1587,13 +1580,13 @@
     </row>
     <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D15" s="9" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A15)</f>
@@ -1608,11 +1601,11 @@
         <v/>
       </c>
       <c r="G15" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A15,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A15,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H15" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A15,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A15,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I15" s="9" t="str">
@@ -1622,13 +1615,13 @@
     </row>
     <row r="16" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D16" s="6" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A16)</f>
@@ -1643,11 +1636,11 @@
         <v/>
       </c>
       <c r="G16" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A16,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A16,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H16" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A16,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A16,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I16" s="6" t="str">
@@ -1657,13 +1650,13 @@
     </row>
     <row r="17" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D17" s="9" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A17)</f>
@@ -1678,11 +1671,11 @@
         <v/>
       </c>
       <c r="G17" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A17,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A17,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H17" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A17,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A17,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I17" s="9" t="str">
@@ -1692,13 +1685,13 @@
     </row>
     <row r="18" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D18" s="6" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A18)</f>
@@ -1713,11 +1706,11 @@
         <v/>
       </c>
       <c r="G18" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A18,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A18,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H18" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A18,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A18,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I18" s="6" t="str">
@@ -1727,13 +1720,13 @@
     </row>
     <row r="19" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D19" s="9" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A19)</f>
@@ -1748,11 +1741,11 @@
         <v/>
       </c>
       <c r="G19" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A19,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A19,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H19" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A19,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A19,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I19" s="9" t="str">
@@ -1762,13 +1755,13 @@
     </row>
     <row r="20" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D20" s="6" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A20)</f>
@@ -1783,11 +1776,11 @@
         <v/>
       </c>
       <c r="G20" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A20,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A20,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H20" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A20,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A20,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I20" s="6" t="str">
@@ -1797,13 +1790,13 @@
     </row>
     <row r="21" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D21" s="9" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A21)</f>
@@ -1818,11 +1811,11 @@
         <v/>
       </c>
       <c r="G21" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A21,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A21,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H21" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A21,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A21,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I21" s="9" t="str">
@@ -1832,13 +1825,13 @@
     </row>
     <row r="22" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D22" s="6" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A22)</f>
@@ -1853,11 +1846,11 @@
         <v/>
       </c>
       <c r="G22" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A22,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A22,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H22" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A22,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A22,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I22" s="6" t="str">
@@ -1867,13 +1860,13 @@
     </row>
     <row r="23" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A23)</f>
@@ -1888,11 +1881,11 @@
         <v/>
       </c>
       <c r="G23" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A23,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A23,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H23" s="9" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A23,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A23,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I23" s="9" t="str">
@@ -1902,13 +1895,13 @@
     </row>
     <row r="24" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D24" s="6" t="n">
         <f aca="false">COUNTIF('Daily Log'!$D$2:$D$31,$A24)</f>
@@ -1923,11 +1916,11 @@
         <v/>
       </c>
       <c r="G24" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A24,'Daily Log'!$J$2:$J$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A24,'Daily Log'!$I$2:$I$31)</f>
         <v>0</v>
       </c>
       <c r="H24" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A24,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$D$2:$D$31,$A24,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="I24" s="6" t="str">
@@ -1962,7 +1955,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -1971,69 +1964,51 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="9" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="14" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="N1" s="5" t="s">
         <v>91</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="R1" s="5" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2044,13 +2019,13 @@
         <v>46239</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F2" s="13"/>
       <c r="G2" s="13"/>
@@ -2059,13 +2034,8 @@
       <c r="J2" s="13"/>
       <c r="K2" s="13"/>
       <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="13"/>
-      <c r="P2" s="13"/>
-      <c r="Q2" s="13"/>
-      <c r="R2" s="14" t="s">
-        <v>98</v>
+      <c r="M2" s="14" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2077,13 +2047,13 @@
         <v>46240</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
@@ -2092,12 +2062,7 @@
       <c r="J3" s="13"/>
       <c r="K3" s="13"/>
       <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="13"/>
-      <c r="R3" s="12"/>
+      <c r="M3" s="12"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="n">
@@ -2108,13 +2073,13 @@
         <v>46241</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
@@ -2123,12 +2088,7 @@
       <c r="J4" s="13"/>
       <c r="K4" s="13"/>
       <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="12"/>
+      <c r="M4" s="12"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="n">
@@ -2139,13 +2099,13 @@
         <v>46242</v>
       </c>
       <c r="C5" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="E5" s="12" t="s">
         <v>96</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>100</v>
       </c>
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
@@ -2154,12 +2114,7 @@
       <c r="J5" s="13"/>
       <c r="K5" s="13"/>
       <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
-      <c r="N5" s="13"/>
-      <c r="O5" s="13"/>
-      <c r="P5" s="13"/>
-      <c r="Q5" s="13"/>
-      <c r="R5" s="12"/>
+      <c r="M5" s="12"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="n">
@@ -2170,13 +2125,13 @@
         <v>46243</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F6" s="13"/>
       <c r="G6" s="13"/>
@@ -2185,12 +2140,7 @@
       <c r="J6" s="13"/>
       <c r="K6" s="13"/>
       <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="13"/>
-      <c r="R6" s="12"/>
+      <c r="M6" s="12"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="n">
@@ -2201,13 +2151,13 @@
         <v>46244</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
@@ -2216,12 +2166,7 @@
       <c r="J7" s="13"/>
       <c r="K7" s="13"/>
       <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="13"/>
-      <c r="Q7" s="13"/>
-      <c r="R7" s="12"/>
+      <c r="M7" s="12"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="n">
@@ -2232,15 +2177,15 @@
         <v>46245</v>
       </c>
       <c r="C8" s="18" t="str">
-        <f aca="false">IFERROR(INDEX(C2:C7,MATCH(MAX(L2:L7),L2:L7,0)),"TBD - no DMs logged yet")</f>
+        <f aca="false">IFERROR(INDEX(C2:C7,MATCH(MAX(K2:K7),K2:K7,0)),"TBD - no DMs logged yet")</f>
         <v>TBD - no DMs logged yet</v>
       </c>
       <c r="D8" s="18" t="str">
-        <f aca="false">IFERROR(INDEX(D2:D7,MATCH(MAX(L2:L7),L2:L7,0)),"TBD - no DMs logged yet")</f>
+        <f aca="false">IFERROR(INDEX(D2:D7,MATCH(MAX(K2:K7),K2:K7,0)),"TBD - no DMs logged yet")</f>
         <v>TBD - no DMs logged yet</v>
       </c>
       <c r="E8" s="18" t="str">
-        <f aca="false">IFERROR(INDEX(E2:E7,MATCH(MAX(L2:L7),L2:L7,0)),"TBD - no DMs logged yet")</f>
+        <f aca="false">IFERROR(INDEX(E2:E7,MATCH(MAX(K2:K7),K2:K7,0)),"TBD - no DMs logged yet")</f>
         <v>TBD - no DMs logged yet</v>
       </c>
       <c r="F8" s="13"/>
@@ -2250,12 +2195,7 @@
       <c r="J8" s="13"/>
       <c r="K8" s="13"/>
       <c r="L8" s="13"/>
-      <c r="M8" s="13"/>
-      <c r="N8" s="13"/>
-      <c r="O8" s="13"/>
-      <c r="P8" s="13"/>
-      <c r="Q8" s="13"/>
-      <c r="R8" s="12"/>
+      <c r="M8" s="12"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="n">
@@ -2275,12 +2215,7 @@
       <c r="J9" s="13"/>
       <c r="K9" s="13"/>
       <c r="L9" s="13"/>
-      <c r="M9" s="13"/>
-      <c r="N9" s="13"/>
-      <c r="O9" s="13"/>
-      <c r="P9" s="13"/>
-      <c r="Q9" s="13"/>
-      <c r="R9" s="12"/>
+      <c r="M9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="n">
@@ -2300,12 +2235,7 @@
       <c r="J10" s="13"/>
       <c r="K10" s="13"/>
       <c r="L10" s="13"/>
-      <c r="M10" s="13"/>
-      <c r="N10" s="13"/>
-      <c r="O10" s="13"/>
-      <c r="P10" s="13"/>
-      <c r="Q10" s="13"/>
-      <c r="R10" s="12"/>
+      <c r="M10" s="12"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="n">
@@ -2325,12 +2255,7 @@
       <c r="J11" s="13"/>
       <c r="K11" s="13"/>
       <c r="L11" s="13"/>
-      <c r="M11" s="13"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="13"/>
-      <c r="Q11" s="13"/>
-      <c r="R11" s="12"/>
+      <c r="M11" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="n">
@@ -2350,12 +2275,7 @@
       <c r="J12" s="13"/>
       <c r="K12" s="13"/>
       <c r="L12" s="13"/>
-      <c r="M12" s="13"/>
-      <c r="N12" s="13"/>
-      <c r="O12" s="13"/>
-      <c r="P12" s="13"/>
-      <c r="Q12" s="13"/>
-      <c r="R12" s="12"/>
+      <c r="M12" s="12"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="n">
@@ -2375,12 +2295,7 @@
       <c r="J13" s="13"/>
       <c r="K13" s="13"/>
       <c r="L13" s="13"/>
-      <c r="M13" s="13"/>
-      <c r="N13" s="13"/>
-      <c r="O13" s="13"/>
-      <c r="P13" s="13"/>
-      <c r="Q13" s="13"/>
-      <c r="R13" s="12"/>
+      <c r="M13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="n">
@@ -2400,12 +2315,7 @@
       <c r="J14" s="13"/>
       <c r="K14" s="13"/>
       <c r="L14" s="13"/>
-      <c r="M14" s="13"/>
-      <c r="N14" s="13"/>
-      <c r="O14" s="13"/>
-      <c r="P14" s="13"/>
-      <c r="Q14" s="13"/>
-      <c r="R14" s="12"/>
+      <c r="M14" s="12"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="n">
@@ -2425,12 +2335,7 @@
       <c r="J15" s="13"/>
       <c r="K15" s="13"/>
       <c r="L15" s="13"/>
-      <c r="M15" s="13"/>
-      <c r="N15" s="13"/>
-      <c r="O15" s="13"/>
-      <c r="P15" s="13"/>
-      <c r="Q15" s="13"/>
-      <c r="R15" s="12"/>
+      <c r="M15" s="12"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="n">
@@ -2450,12 +2355,7 @@
       <c r="J16" s="13"/>
       <c r="K16" s="13"/>
       <c r="L16" s="13"/>
-      <c r="M16" s="13"/>
-      <c r="N16" s="13"/>
-      <c r="O16" s="13"/>
-      <c r="P16" s="13"/>
-      <c r="Q16" s="13"/>
-      <c r="R16" s="12"/>
+      <c r="M16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="n">
@@ -2475,12 +2375,7 @@
       <c r="J17" s="13"/>
       <c r="K17" s="13"/>
       <c r="L17" s="13"/>
-      <c r="M17" s="13"/>
-      <c r="N17" s="13"/>
-      <c r="O17" s="13"/>
-      <c r="P17" s="13"/>
-      <c r="Q17" s="13"/>
-      <c r="R17" s="12"/>
+      <c r="M17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="n">
@@ -2500,12 +2395,7 @@
       <c r="J18" s="13"/>
       <c r="K18" s="13"/>
       <c r="L18" s="13"/>
-      <c r="M18" s="13"/>
-      <c r="N18" s="13"/>
-      <c r="O18" s="13"/>
-      <c r="P18" s="13"/>
-      <c r="Q18" s="13"/>
-      <c r="R18" s="12"/>
+      <c r="M18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="n">
@@ -2525,12 +2415,7 @@
       <c r="J19" s="13"/>
       <c r="K19" s="13"/>
       <c r="L19" s="13"/>
-      <c r="M19" s="13"/>
-      <c r="N19" s="13"/>
-      <c r="O19" s="13"/>
-      <c r="P19" s="13"/>
-      <c r="Q19" s="13"/>
-      <c r="R19" s="12"/>
+      <c r="M19" s="12"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="n">
@@ -2550,12 +2435,7 @@
       <c r="J20" s="13"/>
       <c r="K20" s="13"/>
       <c r="L20" s="13"/>
-      <c r="M20" s="13"/>
-      <c r="N20" s="13"/>
-      <c r="O20" s="13"/>
-      <c r="P20" s="13"/>
-      <c r="Q20" s="13"/>
-      <c r="R20" s="12"/>
+      <c r="M20" s="12"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="n">
@@ -2575,12 +2455,7 @@
       <c r="J21" s="13"/>
       <c r="K21" s="13"/>
       <c r="L21" s="13"/>
-      <c r="M21" s="13"/>
-      <c r="N21" s="13"/>
-      <c r="O21" s="13"/>
-      <c r="P21" s="13"/>
-      <c r="Q21" s="13"/>
-      <c r="R21" s="12"/>
+      <c r="M21" s="12"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="n">
@@ -2600,12 +2475,7 @@
       <c r="J22" s="13"/>
       <c r="K22" s="13"/>
       <c r="L22" s="13"/>
-      <c r="M22" s="13"/>
-      <c r="N22" s="13"/>
-      <c r="O22" s="13"/>
-      <c r="P22" s="13"/>
-      <c r="Q22" s="13"/>
-      <c r="R22" s="12"/>
+      <c r="M22" s="12"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="n">
@@ -2625,12 +2495,7 @@
       <c r="J23" s="13"/>
       <c r="K23" s="13"/>
       <c r="L23" s="13"/>
-      <c r="M23" s="13"/>
-      <c r="N23" s="13"/>
-      <c r="O23" s="13"/>
-      <c r="P23" s="13"/>
-      <c r="Q23" s="13"/>
-      <c r="R23" s="12"/>
+      <c r="M23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="n">
@@ -2650,12 +2515,7 @@
       <c r="J24" s="13"/>
       <c r="K24" s="13"/>
       <c r="L24" s="13"/>
-      <c r="M24" s="13"/>
-      <c r="N24" s="13"/>
-      <c r="O24" s="13"/>
-      <c r="P24" s="13"/>
-      <c r="Q24" s="13"/>
-      <c r="R24" s="12"/>
+      <c r="M24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="n">
@@ -2675,12 +2535,7 @@
       <c r="J25" s="13"/>
       <c r="K25" s="13"/>
       <c r="L25" s="13"/>
-      <c r="M25" s="13"/>
-      <c r="N25" s="13"/>
-      <c r="O25" s="13"/>
-      <c r="P25" s="13"/>
-      <c r="Q25" s="13"/>
-      <c r="R25" s="12"/>
+      <c r="M25" s="12"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="n">
@@ -2700,12 +2555,7 @@
       <c r="J26" s="13"/>
       <c r="K26" s="13"/>
       <c r="L26" s="13"/>
-      <c r="M26" s="13"/>
-      <c r="N26" s="13"/>
-      <c r="O26" s="13"/>
-      <c r="P26" s="13"/>
-      <c r="Q26" s="13"/>
-      <c r="R26" s="12"/>
+      <c r="M26" s="12"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="n">
@@ -2725,12 +2575,7 @@
       <c r="J27" s="13"/>
       <c r="K27" s="13"/>
       <c r="L27" s="13"/>
-      <c r="M27" s="13"/>
-      <c r="N27" s="13"/>
-      <c r="O27" s="13"/>
-      <c r="P27" s="13"/>
-      <c r="Q27" s="13"/>
-      <c r="R27" s="12"/>
+      <c r="M27" s="12"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="n">
@@ -2750,12 +2595,7 @@
       <c r="J28" s="13"/>
       <c r="K28" s="13"/>
       <c r="L28" s="13"/>
-      <c r="M28" s="13"/>
-      <c r="N28" s="13"/>
-      <c r="O28" s="13"/>
-      <c r="P28" s="13"/>
-      <c r="Q28" s="13"/>
-      <c r="R28" s="12"/>
+      <c r="M28" s="12"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="n">
@@ -2775,12 +2615,7 @@
       <c r="J29" s="13"/>
       <c r="K29" s="13"/>
       <c r="L29" s="13"/>
-      <c r="M29" s="13"/>
-      <c r="N29" s="13"/>
-      <c r="O29" s="13"/>
-      <c r="P29" s="13"/>
-      <c r="Q29" s="13"/>
-      <c r="R29" s="12"/>
+      <c r="M29" s="12"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="n">
@@ -2800,12 +2635,7 @@
       <c r="J30" s="13"/>
       <c r="K30" s="13"/>
       <c r="L30" s="13"/>
-      <c r="M30" s="13"/>
-      <c r="N30" s="13"/>
-      <c r="O30" s="13"/>
-      <c r="P30" s="13"/>
-      <c r="Q30" s="13"/>
-      <c r="R30" s="12"/>
+      <c r="M30" s="12"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="n">
@@ -2825,12 +2655,7 @@
       <c r="J31" s="13"/>
       <c r="K31" s="13"/>
       <c r="L31" s="13"/>
-      <c r="M31" s="13"/>
-      <c r="N31" s="13"/>
-      <c r="O31" s="13"/>
-      <c r="P31" s="13"/>
-      <c r="Q31" s="13"/>
-      <c r="R31" s="12"/>
+      <c r="M31" s="12"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2861,33 +2686,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C2" s="6" t="str">
         <f aca="false">IFERROR(AVERAGEIF('Daily Log'!$C$2:$C$31,$A2,'Daily Log'!$F$2:$F$31),"")</f>
@@ -2898,11 +2723,11 @@
         <v/>
       </c>
       <c r="E2" s="6" t="str">
-        <f aca="false">IFERROR(AVERAGEIF('Daily Log'!$C$2:$C$31,$A2,'Daily Log'!$J$2:$J$31),"")</f>
+        <f aca="false">IFERROR(AVERAGEIF('Daily Log'!$C$2:$C$31,$A2,'Daily Log'!$I$2:$I$31),"")</f>
         <v/>
       </c>
       <c r="F2" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$C$2:$C$31,$A2,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$C$2:$C$31,$A2,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="G2" s="6" t="str">
@@ -2912,10 +2737,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C3" s="6" t="str">
         <f aca="false">IFERROR(AVERAGEIF('Daily Log'!$C$2:$C$31,$A3,'Daily Log'!$F$2:$F$31),"")</f>
@@ -2926,11 +2751,11 @@
         <v/>
       </c>
       <c r="E3" s="6" t="str">
-        <f aca="false">IFERROR(AVERAGEIF('Daily Log'!$C$2:$C$31,$A3,'Daily Log'!$J$2:$J$31),"")</f>
+        <f aca="false">IFERROR(AVERAGEIF('Daily Log'!$C$2:$C$31,$A3,'Daily Log'!$I$2:$I$31),"")</f>
         <v/>
       </c>
       <c r="F3" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$C$2:$C$31,$A3,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$C$2:$C$31,$A3,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="G3" s="6" t="str">
@@ -2940,10 +2765,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C4" s="6" t="str">
         <f aca="false">IFERROR(AVERAGEIF('Daily Log'!$C$2:$C$31,$A4,'Daily Log'!$F$2:$F$31),"")</f>
@@ -2954,11 +2779,11 @@
         <v/>
       </c>
       <c r="E4" s="6" t="str">
-        <f aca="false">IFERROR(AVERAGEIF('Daily Log'!$C$2:$C$31,$A4,'Daily Log'!$J$2:$J$31),"")</f>
+        <f aca="false">IFERROR(AVERAGEIF('Daily Log'!$C$2:$C$31,$A4,'Daily Log'!$I$2:$I$31),"")</f>
         <v/>
       </c>
       <c r="F4" s="6" t="n">
-        <f aca="false">SUMIF('Daily Log'!$C$2:$C$31,$A4,'Daily Log'!$L$2:$L$31)</f>
+        <f aca="false">SUMIF('Daily Log'!$C$2:$C$31,$A4,'Daily Log'!$K$2:$K$31)</f>
         <v>0</v>
       </c>
       <c r="G4" s="6" t="str">
@@ -2968,7 +2793,7 @@
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B6" s="19"/>
       <c r="C6" s="19"/>
@@ -3010,18 +2835,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="19" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B2" s="19"/>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="20" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B4" s="18" t="n">
         <f aca="false">SUM('Daily Log'!F2:F8)</f>
@@ -3030,16 +2855,16 @@
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B5" s="18" t="n">
-        <f aca="false">SUM('Daily Log'!I2:I8)+SUM('Daily Log'!J2:J8)+SUM('Daily Log'!K2:K8)+SUM('Daily Log'!M2:M8)</f>
+        <f aca="false">SUM('Daily Log'!H2:H8)+SUM('Daily Log'!I2:I8)+SUM('Daily Log'!J2:J8)+SUM('Daily Log'!L2:L8)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B6" s="21" t="str">
         <f aca="false">IFERROR(B5/B4*100,"")</f>
@@ -3048,22 +2873,22 @@
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B7" s="18" t="n">
-        <f aca="false">SUM('Daily Log'!L2:L8)</f>
+        <f aca="false">SUM('Daily Log'!K2:K8)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B8" s="12"/>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B9" s="18" t="str">
         <f aca="false">IFERROR(AVERAGE('Daily Log'!G2:G8),"")</f>
@@ -3072,7 +2897,7 @@
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B10" s="18" t="str">
         <f aca="false">IFERROR(INDEX('Format Comparison'!B2:B4,MATCH("Winner (most DMs)",'Format Comparison'!G2:G4,0)),"TBD -- need more data")</f>
@@ -3081,7 +2906,7 @@
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B11" s="18" t="str">
         <f aca="false">IF(SUM('Hook Bank'!H2:H24)=0,"TBD -- need more data",INDEX('Hook Bank'!A2:A24,MATCH(MAX('Hook Bank'!H2:H24),'Hook Bank'!H2:H24,0)))</f>
@@ -3090,7 +2915,7 @@
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B12" s="18" t="str">
         <f aca="false">IF(SUM('Hook Bank'!H2:H24)=0,"TBD",INDEX('Hook Bank'!C2:C24,MATCH(MAX('Hook Bank'!H2:H24),'Hook Bank'!H2:H24,0)))</f>
@@ -3099,7 +2924,7 @@
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B13" s="18" t="str">
         <f aca="false">IFERROR(('Daily Log'!F8-'Daily Log'!F2)/'Daily Log'!F2*100,"")</f>
@@ -3108,7 +2933,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>